<commit_message>
Auto export Excel 2026-06-21
</commit_message>
<xml_diff>
--- a/exports/history_export_in.xlsx
+++ b/exports/history_export_in.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
   <si>
     <t>ลำดับ</t>
   </si>
@@ -49,16 +49,10 @@
     <t/>
   </si>
   <si>
-    <t>Service</t>
-  </si>
-  <si>
-    <t>2026-06-21 13:37:49</t>
-  </si>
-  <si>
     <t>Install</t>
   </si>
   <si>
-    <t>2026-06-21 13:37:38</t>
+    <t>2026-06-21 13:42:14</t>
   </si>
 </sst>
 </file>
@@ -81,7 +75,7 @@
       <color rgb="FFE8EAF0"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -96,11 +90,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF181C27"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F2435"/>
       </patternFill>
     </fill>
   </fills>
@@ -125,15 +114,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -475,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -538,7 +524,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>11</v>
@@ -551,38 +537,6 @@
       </c>
       <c r="J2" s="2" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="3">
-        <v>4</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>